<commit_message>
Add species status: Amazona oratrix -> False Positive
</commit_message>
<xml_diff>
--- a/UK_Birds_Generalized_Status.xlsx
+++ b/UK_Birds_Generalized_Status.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C649"/>
+  <dimension ref="A1:C650"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="25" bestFit="1" customWidth="1" min="1" max="2"/>
@@ -11514,6 +11514,23 @@
         </is>
       </c>
     </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>Yellow-headed Parrot</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>Amazona oratrix</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>False Positive</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>